<commit_message>
new dark icons & breakthrough fixes
</commit_message>
<xml_diff>
--- a/Template_Data.xlsx
+++ b/Template_Data.xlsx
@@ -1015,7 +1015,7 @@
     <t>Bentor</t>
   </si>
   <si>
-    <t>&lt;fs=64&gt;Кокнлав историков&lt;/fs&gt;</t>
+    <t>&lt;fs=64&gt;Конклав историков&lt;/fs&gt;</t>
   </si>
   <si>
     <t>&lt;fc=CF14EE&gt;&lt;fs=40&gt;Бенторийский Конгломерат&lt;/fs&gt;&lt;/fc&gt;</t>
@@ -1147,7 +1147,7 @@
     <t>&lt;fc=F1B823&gt;&lt;fs=30&gt;Горнодобывающий консорциум «ПРГ»&lt;/fs&gt;&lt;/fc&gt;</t>
   </si>
   <si>
-    <t>&lt;f=Myriad Pro Light;50;1;0;0;0&gt;&lt;ls=75&gt;&lt;push=0;50&gt;Подконтрольные вам планеты с размещённом на ней жетоном ядра считатся станциями (кроме установления контроля).&lt;/ls&gt;&lt;ls=60&gt;&lt;br&gt;&lt;br&gt;&lt;/ls&gt;&lt;ls=75&gt;Подконтрольные вам станции получают способность &lt;/f&gt;&lt;push=0;17&gt;&lt;f=Russo One;40;0;0;0;0&gt;«КОСМИЧЕСКАЯ ПУШКА 5»&lt;/f&gt;&lt;push=0;-17&gt;&lt;f=Myriad Pro Light;50;1;0;0;0&gt;.&lt;/ls&gt;&lt;/f&gt;</t>
+    <t>&lt;f=Myriad Pro Light;50;1;0;0;0&gt;&lt;ls=75&gt;&lt;push=0;50&gt;Подконтрольные вам планеты с размещённом на ней жетоном ядра считаются станциями (кроме установления контроля).&lt;/ls&gt;&lt;ls=60&gt;&lt;br&gt;&lt;br&gt;&lt;/ls&gt;&lt;ls=75&gt;Подконтрольные вам станции получают способность &lt;/f&gt;&lt;push=0;17&gt;&lt;f=Russo One;40;0;0;0;0&gt;«КОСМИЧЕСКАЯ ПУШКА 5»&lt;/f&gt;&lt;push=0;-17&gt;&lt;f=Myriad Pro Light;50;1;0;0;0&gt;.&lt;/ls&gt;&lt;/f&gt;</t>
   </si>
   <si>
     <t>Ilyxum</t>
@@ -1213,7 +1213,7 @@
     <t>Kyro</t>
   </si>
   <si>
-    <t>&lt;fs=64&gt;Расространение штамма&lt;/fs&gt;</t>
+    <t>&lt;fs=64&gt;Распространение штамма&lt;/fs&gt;</t>
   </si>
   <si>
     <t>&lt;fc=B0DE1C&gt;&lt;fs=40&gt;Община Кайро&lt;/fs&gt;&lt;/fc&gt;</t>

</xml_diff>